<commit_message>
Style and document the Excel lead export
The export was plain pandas output: no header fill, default column
widths, no frozen pane. Give the workbook a bold green header, a frozen
top row, content-fit column widths, an auto-filter, and banded rows so
the delivered file looks finished and a README screenshot can show it
honestly.

Cover the styling with tests, restyle the committed samples through the
new export, add a docs/ screenshot, and note the DuckDuckGo throttle
limit plus the keyed-search-API path under a Limitations section.
</commit_message>
<xml_diff>
--- a/samples/wy_large_carriers.xlsx
+++ b/samples/wy_large_carriers.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Leads" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="QA Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$K$45</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +28,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00217346"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF3EF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,59 +434,72 @@
   </sheetPr>
   <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DOT#</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Street</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ZIP</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Power units</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Trucks</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Drivers</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
@@ -522,47 +553,47 @@
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>52081</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>WYOMING MACHINERY COMPANY</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>5300 WEST OLD YELLOWSTONE HWY</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>CASPER</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>82604</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="2" t="n">
         <v>181</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="2" t="n">
         <v>168</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="2" t="n">
         <v>179</v>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -612,51 +643,51 @@
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>100378</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>JOHN BUNNING TRANSFER COMPANY INC</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>(307) 362-3791</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>1600 ELK ST</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>ROCK SPRINGS</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>82901-4021</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>MOLTEN SULFUR</t>
         </is>
@@ -710,51 +741,51 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>104367</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>SIMON CONTRACTORS</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>(307) 632-7900</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>4819 S INDUSTRIAL SERVICE RD</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>CHEYENNE</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>82007</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="2" t="n">
         <v>103</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>ROAD BUILDING MATERIAL</t>
         </is>
@@ -808,51 +839,51 @@
       <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>155142</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>ADMIRAL TRANSPORT CORPORATION</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>(307) 278-2024</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>821 PULLIAM</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>WORLAND</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>82401</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="2" t="n">
         <v>519</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="2" t="n">
         <v>516</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="2" t="n">
         <v>849</v>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -902,47 +933,47 @@
       <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>254966</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>HIGH WEST ENERGY INC</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>6270 RD 212</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>PINE BLUFFS</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>82082</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>TOOLS</t>
         </is>
@@ -1000,51 +1031,51 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>288449</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>GK CONSTRUCTION INC</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>(307) 548-6155</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>1169 LANE 11 1/2</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>LOVELL</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>82431-9547</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>BENTONITE, AGGREGATE</t>
         </is>
@@ -1102,51 +1133,51 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>345250</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>BLAKEMAN PROPANE INC</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>(307) 756-3302</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>801 W CONVERSE ST</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>MOORCROFT</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>82721</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1200,51 +1231,51 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>381386</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>TETON DISTRIBUTORS INC</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>(307) 278-2776</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>821 PULLIAM</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>WORLAND</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>82401</t>
         </is>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="2" t="n">
         <v>86</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1298,47 +1329,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>472709</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>DESERT MOUNTAIN CORPORATION</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>2095 CHANDELLE</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>RIVERTON</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>82501</t>
         </is>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1388,51 +1419,51 @@
       <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>535361</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>CITY OF CASPER</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>(307) 235-8392</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>1800 EAST K ST</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>CASPER</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>82601</t>
         </is>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" s="2" t="n">
         <v>124</v>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1482,51 +1513,51 @@
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>546163</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>UNION TELEPHONE COMPANY</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>(307) 782-6131</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>850 HWY 414 N</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>MOUNTAIN VIEW</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>82939</t>
         </is>
       </c>
-      <c r="H23" t="n">
+      <c r="H23" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1580,51 +1611,51 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>863077</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>SCHULTE TA INC</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>(307) 685-3181</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>5950 SWANSON RD</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>GILLETTE</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>82718</t>
         </is>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="J25" t="n">
+      <c r="J25" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1674,51 +1705,51 @@
       <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>1223293</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>WYOMING ENVIRONMENTAL SERVICES</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>(800) 479-9173</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>1754 INTERCHANGE RD</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>ROCK SPRINGS</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>82901</t>
         </is>
       </c>
-      <c r="H27" t="n">
+      <c r="H27" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="J27" t="n">
+      <c r="J27" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>TRASH</t>
         </is>
@@ -1772,51 +1803,51 @@
       <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>1294615</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>ACTION CARGO CORPORATION</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>(307) 266-2229</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>2600 E YELLOWSTONE HIGHWAY</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>CASPER</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>82609</t>
         </is>
       </c>
-      <c r="H29" t="n">
+      <c r="H29" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="J29" t="n">
+      <c r="J29" s="2" t="n">
         <v>107</v>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1870,51 +1901,51 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>1557547</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>HALL TRUCKING INC</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>(307) 273-4000</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>6700 EAST YELLOWSTONE ROAD</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>EVANSVILLE</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>82636</t>
         </is>
       </c>
-      <c r="H31" t="n">
+      <c r="H31" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="I31" t="n">
+      <c r="I31" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="J31" t="n">
+      <c r="J31" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1964,51 +1995,51 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>2131618</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>R&amp;R SERVICES INC</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>(307) 462-2900</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>30 S JAMES FAIRBANKS LN</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>BOULDER</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>82923</t>
         </is>
       </c>
-      <c r="H33" t="n">
+      <c r="H33" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="J33" t="n">
+      <c r="J33" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2058,51 +2089,51 @@
       <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>2170456</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>PRAIRIE FIELD SERVICES LLC</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>(952) 345-8911</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>3019 SALT CREEK HIGHWAY</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>CASPER</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>82601</t>
         </is>
       </c>
-      <c r="H35" t="n">
+      <c r="H35" s="2" t="n">
         <v>113</v>
       </c>
-      <c r="I35" t="n">
+      <c r="I35" s="2" t="n">
         <v>113</v>
       </c>
-      <c r="J35" t="n">
+      <c r="J35" s="2" t="n">
         <v>117</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2148,47 +2179,47 @@
       <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>2575354</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>WALKER INSPECTION LLC</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>1401 ECHETA ROAD</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>GILLETE</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>82716</t>
         </is>
       </c>
-      <c r="H37" t="n">
+      <c r="H37" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I37" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="J37" t="n">
+      <c r="J37" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2238,51 +2269,51 @@
       <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>3240911</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>ELEMENT TECHINCAL SERVICES LLC</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>(403) 930-0249</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>675 HERFORD LANE</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>CASPER</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>82609</t>
         </is>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2332,51 +2363,51 @@
       <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>3423385</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>PARADISE EXPRESS INC</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>(888) 537-0558</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>4200 S POPLAR STREET SUITE 5</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>CASPER</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>82601</t>
         </is>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I41" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="J41" t="n">
+      <c r="J41" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2422,47 +2453,47 @@
       <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>4251471</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>VISIONARY COMMUNICATIONS LLC</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>1001 S DOUGLAS HWY STE 201</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>GILLETTE</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>82716-4957</t>
         </is>
       </c>
-      <c r="H43" t="n">
+      <c r="H43" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" s="2" t="n">
         <v>87</v>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2512,53 +2543,54 @@
       <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>4498390</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>TM NATIONS LOGISTICS LLC</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>(307) 922-4705</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>295 GANNETT DR</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>ROCK SPRINGS</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>WY</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>82901</t>
         </is>
       </c>
-      <c r="H45" t="n">
+      <c r="H45" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I45" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2571,14 +2603,18 @@
   </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>

</xml_diff>